<commit_message>
Finish solo Sankalpam without in-repo audio, and drop the unused design copy from content.
Recordings will arrive from Sarvam later. Until then the player counts with Done and the ring, the Ganesha drawings are in the pack, and content/sankalpam is removed because those files already live in docs/.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M1-sankalpam.xlsx
+++ b/tests/M1-sankalpam.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -454,6 +454,7 @@
     <col width="24.140625" customWidth="1" min="7" max="7"/>
     <col width="26.5703125" customWidth="1" min="8" max="8"/>
     <col width="30.42578125" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +513,11 @@
           <t>Test Type</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="57.95" customHeight="1">
       <c r="A2" s="3" t="n">
@@ -556,6 +562,11 @@
       </c>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>PASS. build_content.py --check: 0 errors, 0 warnings, 108 names. Flags: 10 VARIANT; 36, 37, 40, 73, 75, 81, 86, 98, 105 CORRECTED; 65, 77, 103 SCRIPT; 108 VARIANT.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="57.95" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -602,6 +613,11 @@
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>PASS. The player opened. My japam showed Ganapati mula mantra, 0 so far, of 10,008, Day 1 of 41.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.95" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -647,6 +663,11 @@
       </c>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>PASS. On step 3 with no text, Start is not clickable and the form shows Choose what you will chant.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.95" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -692,6 +713,11 @@
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>PASS. The reason appears only in About, as “for my mother health · only you see this”. It is not on the card or on Home. The apostrophe did not survive the emulator keyboard.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="57.95" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -737,6 +763,11 @@
       </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="57.95" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -782,6 +813,11 @@
       </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="57.95" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -827,6 +863,11 @@
       </c>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.95" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -872,6 +913,11 @@
       </c>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="57.95" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -917,6 +963,11 @@
       </c>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="57.95" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -962,6 +1013,11 @@
       </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="57.95" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1007,6 +1063,11 @@
       </c>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="57.95" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1052,6 +1113,11 @@
       </c>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="57.95" customHeight="1">
       <c r="A14" s="3" t="n">
@@ -1097,6 +1163,11 @@
       </c>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="57.95" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1142,6 +1213,11 @@
       </c>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="57.95" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1187,6 +1263,11 @@
       </c>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>PASS. Added 3 for Sun 20 Sep on the 11-day aṣṭottaram. About showed that day, 3, and added by hand.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="57.95" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -1232,6 +1313,11 @@
       </c>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>PASS. The day chips run from Today back through the start day (Mon 14) and no earlier. At 0 the sheet stays open and the button stays Add 0.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="57.95" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -1277,6 +1363,11 @@
       </c>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>PASS. After 3 the line was Goal reached · 3 · keep chanting. After 2 more the card showed 5 so far · of 3. Reopening showed Today 5 · Total 5 of 3, and the goal line did not return.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="57.95" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -1322,6 +1413,11 @@
       </c>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>PASS. With the debug date on 15 Sep the 1-day japam was under Completed: 0 offered · 1 days · ended Mon 14 Sep. No missed-days wording.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="57.95" customHeight="1">
       <c r="A20" s="3" t="n">
@@ -1367,6 +1463,11 @@
       </c>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>PASS. Start again opened step 3 of 3 for Ganesha Ashtottara, goal 108, Other set to 1, and Today as the start. Start was not tapped.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="57.95" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -1411,6 +1512,11 @@
       </c>
       <c r="J21" s="4" t="inlineStr"/>
       <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Debug build: the pack has no audio file. The aṣṭottaram shows Done and no Play. The mantra shows the ring only and no Play. A release APK was not installed.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="57.95" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -1456,6 +1562,11 @@
       </c>
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>PASS offline: cold start, the player, a ring tap (88 to 89) and Add 1 by hand all worked, with no connection message. Play is waiting for audio.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="57.95" customHeight="1">
       <c r="A23" s="3" t="n">
@@ -1501,6 +1612,11 @@
       </c>
       <c r="J23" s="4" t="inlineStr"/>
       <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>PASS. On 21 Sep, Home and My japam showed the existing totals and Day 8. No missed days, streaks, 0 today, or red.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>